<commit_message>
Expand patient dataset: add 10 synthetic cases across cardiology, respiratory, gastro, neuro, endocrine, ortho, derm, gynecology, pediatrics, urology
</commit_message>
<xml_diff>
--- a/dataset/patient_text.xlsx
+++ b/dataset/patient_text.xlsx
@@ -1,218 +1,177 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
-  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23400" windowHeight="11655"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="23400" windowHeight="11655" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="病程记录_首次病程" sheetId="3" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="病程记录_首次病程" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
-  <si>
-    <t>Patient-SN</t>
-  </si>
-  <si>
-    <t>case_character</t>
-  </si>
-  <si>
-    <t>treatment_plan</t>
-  </si>
-  <si>
-    <t>00e68831eb28e7bbf58fc289874370bb</t>
-  </si>
-  <si>
-    <t>1、患者。2、缘于1年前患者无意中出现反复咳嗽，无痰，半年前出现右耳闷塞感，未予重视，... 左侧乳突炎。</t>
-  </si>
-  <si>
-    <t>1、完善各项检查，做好治疗前准备。2、予以放化综合治疗。</t>
-  </si>
-</sst>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="20">
     <font>
-      <sz val="11"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF0000FF"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FF800080"/>
+      <sz val="11"/>
+      <u val="single"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
+      <b val="1"/>
+      <color theme="3"/>
       <sz val="18"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <i val="1"/>
+      <color rgb="FF7F7F7F"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <b val="1"/>
       <color theme="3"/>
+      <sz val="15"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
+      <b val="1"/>
       <color theme="3"/>
+      <sz val="13"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
+      <b val="1"/>
       <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <b val="1"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF9C0006"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="宋体"/>
+      <charset val="0"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
+      <sz val="11"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -513,153 +472,153 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -713,11 +672,74 @@
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -1006,39 +1028,223 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="1" outlineLevelCol="2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5" outlineLevelRow="1"/>
   <cols>
-    <col min="1" max="1" width="28.0796460176991" customWidth="1"/>
-    <col min="2" max="2" width="161.884955752212" customWidth="1"/>
+    <col width="28.0796460176991" customWidth="1" min="1" max="1"/>
+    <col width="161.884955752212" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>2</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Patient-SN</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>case_character</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>treatment_plan</t>
+        </is>
       </c>
     </row>
-    <row r="2" spans="1:3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>00e68831eb28e7bbf58fc289874370bb</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1、患者。2、缘于1年前患者无意中出现反复咳嗽，无痰，半年前出现右耳闷塞感，未予重视，... 左侧乳突炎。</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>1、完善各项检查，做好治疗前准备。2、予以放化综合治疗。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>4a26a585bec090ff0339009d25f64042</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1、患者，男性，62岁。2、缘于2年前患者无明显诱因出现活动后胸闷、气短，休息后可缓解，近3个月症状加重，伴心前区压榨样疼痛，向左肩放射，每次持续3-5分钟，含服硝酸甘油后可缓解。既往高血压病史10年，最高180/100mmHg，服用硝苯地平控释片降压，血压控制欠佳。吸烟史40年，每日20支。3、心电图示：V1-V4导联ST段下移0.1mV，T波倒置。心脏超声示：左室舒张功能减退，EF 52%。冠脉CTA示：前降支中段管腔狭窄约70%。</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1、冠脉造影检查，明确冠脉病变程度及范围，必要时行PCI术。2、优化药物治疗：阿司匹林+替格瑞洛双抗，阿托伐他汀调脂，美托洛尔控制心率，硝苯地平控释片联合厄贝沙坦控制血压。3、戒烟，低盐低脂饮食，适度有氧运动。</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ae4f7d3ca8b13c140ceea4ce0cb7848f</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1、患者，女性，35岁。2、缘于5天前受凉后出现发热，体温最高39.2℃，伴畏寒、咳嗽、咳黄色黏痰，痰量中等，无明显臭味。伴有右侧胸痛，深呼吸及咳嗽时加重。自服头孢类抗生素3天，症状无明显改善。既往体健，无基础疾病。3、查体：T 38.6℃，右肺中下野可闻及湿啰音。血常规示：WBC 14.2×10⁹/L，NEUT% 85%，CRP 86mg/L。胸部CT示：右肺下叶大片状高密度影，边缘模糊，可见支气管充气征。</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1、完善痰培养+药敏检查，指导抗生素选择。2、经验性抗感染治疗：莫西沙星400mg ivgtt qd，联合头孢曲松2g ivgtt qd。3、对症支持：氨溴索祛痰、物理降温、补液。4、治疗48-72h后评估疗效，根据药敏结果调整方案。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>d8bd5e59c8cf2efbf0cf821d843e53c4</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1、患者，男性，45岁。2、缘于1年前出现反复反酸、烧心，胸骨后不适感，多在餐后1-2小时及夜间卧位时加重，坐起或服用铝碳酸镁后可缓解。近2月症状加重，偶有吞咽不畅感及声音嘶哑。既往体健，体型偏胖（BMI 28.3），饮食不规律，喜辛辣及咖啡。3、胃镜检查示：食管下段黏膜充血、糜烂，齿状线上移约2cm，贲门松弛，LA-B级食管炎。幽门螺杆菌呼气试验阴性。</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1、生活方式干预：减重，抬高床头，睡前3小时禁食，避免辛辣、油腻、咖啡、巧克力等诱因。2、药物治疗：艾司奥美拉唑20mg bid 8周，莫沙必利5mg tid。3、8周后复查胃镜评估食管黏膜愈合情况，调整为按需治疗。4、若药物效果不佳，考虑食管测压及24h pH监测，评估手术指征。</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1b8a2f67e9d89e4a1a5918c1bc83c01c</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1、患者，男性，68岁。2、缘于6小时前晨起时突发言语不清、右侧肢体无力，伴口角歪斜，无意识障碍、无头痛呕吐。家属发现后立即送至急诊。既往高血压病史15年、2型糖尿病史8年，长期口服降压降糖药，但用药不规律。有吸烟饮酒史。3、查体：神志清楚，运动性失语，右侧鼻唇沟变浅，右上肢肌力3级，右下肢肌力4级，右侧巴氏征阳性。NIHSS评分8分。急诊头颅CT示：未见明显出血灶，左侧大脑中动脉供血区可见稍低密度影。CTA示：左侧大脑中动脉M1段重度狭窄。</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>1、发病在4.5h内，评估溶栓指征，若符合条件行阿替普酶静脉溶栓。2、抗血小板治疗：阿司匹林+氯吡格雷双抗21天后改为单药。3、阿托伐他汀强化降脂，控制血压于140/90mmHg以下，控制血糖达标。4、早期康复介入：肢体功能训练、言语康复、吞咽功能评估。5、完善头颅MRI+MRA，明确梗死范围及血管狭窄程度。</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>371cbb44a8990d89635f659def8afc71</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>1、患者，女性，55岁。2、缘于发现血糖升高5年，诊断为2型糖尿病，曾口服二甲双胍+格列美脲降糖，近1年血糖控制欠佳，空腹血糖9-12mmol/L，餐后2h血糖14-18mmol/L，HbA1c 8.9%。近半年出现双下肢麻木、刺痛感，以夜间为重，伴视物模糊。既往高血压病史8年，高脂血症史5年。母亲有糖尿病史。3、眼底检查示：双眼糖尿病视网膜病变（非增殖期）。双下肢振动觉、温度觉减退，踝反射减弱。尿微量白蛋白/肌酐比值（UACR）：86mg/g。</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>1、调整降糖方案：二甲双胍缓释片+达格列净+司美格鲁肽注射液，目标空腹血糖&lt;7.0mmol/L，餐后2h&lt;10.0mmol/L，HbA1c&lt;7.0%。2、强化降压调脂：厄贝沙坦+氨氯地平控制血压&lt;130/80mmHg，阿托伐他汀控制LDL-C&lt;1.8mmol/L。3、糖尿病并发症管理：甲钴胺营养神经，羟苯磺酸钙改善微循环，定期眼科随访，每年糖尿病肾病筛查。4、糖尿病自我管理教育：饮食控制、运动处方、血糖监测。</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>daf85c0c1c8ad42aad576b4ee9a5a12e</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>1、患者，男性，40岁。2、缘于3月前搬重物后突发腰痛，后逐渐出现左下肢放射性疼痛，沿臀部→大腿后侧→小腿外侧→足背放射，伴左足背外侧麻木感。咳嗽、打喷嚏时疼痛加重，平卧可减轻。既往长期久坐办公，偶有腰痛。3、查体：腰椎前屈受限，左侧直腿抬高试验阳性（40°），加强试验阳性。左下肢肌力正常，左足背感觉减退。腰椎MRI示：L4/5椎间盘左后突出，压迫左侧L5神经根。</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>1、保守治疗为主：急性期卧床休息3-5天，非甾体抗炎药止痛，甲钴胺营养神经，辅以理疗（中频电疗、腰椎牵引）。2、2周后开始核心肌群康复训练，改善腰椎稳定性。3、若保守治疗6-8周无效或出现进行性肌力下降、马尾神经症状，考虑椎间孔镜下髓核摘除术。4、职业健康指导：避免久坐、弯腰负重，正确姿势搬运。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>03a43fad29ded3b2e713b17f3e5d5661</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>1、患者，女性，28岁。2、缘于2年前无明显诱因头皮出现红色斑块，上覆银白色鳞屑，伴轻度瘙痒。皮损逐渐扩展至四肢伸侧及躯干，呈对称分布。曾在当地诊所用激素药膏治疗，暂时好转但反复发作。近1月因工作压力大，皮损明显加重，累及面积约15%体表面积。情绪焦虑，因外观问题不愿社交。无关节肿痛，无指甲改变。3、皮肤科检查：头皮、四肢伸侧及躯干可见散在分布的大小不等红色斑块，边界清楚，上覆多层银白色鳞屑，Auspitz征阳性。PASI评分12分。</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1、局部治疗：糖皮质激素软膏外用（躯干四肢用强效、面部间擦部位用弱效），联合卡泊三醇软膏交替使用，头皮用激素洗剂。2、光疗：窄谱中波紫外线（NB-UVB）治疗，每周3次，逐渐增加剂量。3、若上述治疗3月效果欠佳，评估系统治疗指征，可选用甲氨蝶呤或生物制剂（司库奇尤单抗等）。4、心理辅导，减轻焦虑，建立慢性病长期管理观念。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>57b98a11e4908bbc3df9ca027bc6934a</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>1、患者，女性，42岁。2、缘于1年前发现月经量明显增多，经期延长至8-10天，周期尚规律。伴有轻度痛经及腰骶部坠胀感。近3月出现头晕、乏力、面色苍白等活动后气促等贫血表现。既往体健，孕2产1，未避孕。3、妇科B超示：子宫前壁肌壁间可见一低回声团，大小约5.8×4.5cm，边界清晰，考虑子宫肌瘤。子宫内膜线后移。血常规示：HGB 82g/L，MCV 72fL，呈小细胞低色素性贫血。</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>1、纠正贫血：琥珀酸亚铁口服补铁，维生素C促进铁吸收。2、药物控制症状：GnRH激动剂术前缩瘤或米非司酮减少出血。3、手术治疗：患者已近围绝经期，肌瘤较大且有压迫症状和贫血，建议行腹腔镜下子宫肌瘤剔除术，术中根据情况决定是否保留子宫。4、术前完善宫颈TCT+HPV筛查，排除宫颈病变。</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>026f48aa341cfe17221df0c25e5abe4e</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>1、患者，男性，7岁。2、缘于2年前开始反复出现发作性喘息、咳嗽，春秋季及夜间症状加重，运动后也可诱发。每次发作时双肺可闻及广泛哮鸣音。曾在当地医院雾化治疗后缓解。近半年发作频率增加，约每月1-2次。既往有婴儿湿疹史，父亲有过敏性鼻炎史。3、查体：神清，呼吸稍促，双肺呼吸音粗，可闻及散在哮鸣音。肺功能示：FEV1/FVC 76%，支气管舒张试验阳性（FEV1改善率15%）。过敏原检测：尘螨+++、花粉+。</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>1、急性发作期：沙丁胺醇雾化吸入，必要时加用异丙托溴铵，严重者口服泼尼松3-5天。2、长期控制：低剂量吸入性糖皮质激素（布地奈德）每日规律使用，联合孟鲁司特钠口服。每3月评估哮喘控制水平，阶梯式调整用药。3、环境控制：防螨处理床上用品、减少室内过敏原，避免被动吸烟。4、家长及患儿教育：哮喘行动计划、峰流速仪使用、吸入技术培训。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>57905af274a55d220e6bddebe684168f</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>1、患者，男性，68岁。2、缘于3年前出现夜尿增多（每夜3-4次），排尿费力，尿线变细，排尿后滴沥。近半年症状加重，出现排尿踌躇、间歇性排尿，有时有尿不尽感。无明显尿痛、血尿。既往体检发现前列腺增生2年，未规律治疗。3、直肠指诊：前列腺Ⅱ度增大，表面光滑，中央沟变浅，质地中等。泌尿系B超示：前列腺大小约5.2×4.8×4.5cm（估重约58g），向膀胱内突出约1.2cm，残余尿量约85ml。PSA 2.8ng/ml。</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>1、药物治疗：坦索罗辛（α1受体阻滞剂）改善排尿症状，联合非那雄胺（5α还原酶抑制剂）缩小前列腺体积，需长期服用。2、定期监测：每6-12月复查PSA、泌尿系B超及残余尿量测定，评估IPSS评分变化。3、若药物治疗效果欠佳或出现反复尿潴留、膀胱结石等并发症，考虑经尿道前列腺电切术（TURP）或其他微创治疗。4、生活方式指导：避免久坐、酒精和咖啡因，合理安排饮水时间。</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>